<commit_message>
Add word counts to Participant responses file
</commit_message>
<xml_diff>
--- a/T1DM Treatment Decision Making/Responses/Participant responses.xlsx
+++ b/T1DM Treatment Decision Making/Responses/Participant responses.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11207"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
   <workbookPr hidePivotFieldList="1"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/user/Desktop/GIMA-T1DM-Dataset/T1DM Treatment Decision Making/Responses/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Vee/Desktop/GIMA-T1DM-Dataset/T1DM Treatment Decision Making/Responses/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E01024EA-E916-CE43-A63A-E937EB535179}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FDF33F2-8F98-5148-AF10-9CBDFC0E59E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17260" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Responses" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Responses!$A$1:$S$87</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Responses!$A$1:$T$87</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35,8 +35,30 @@
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1369" uniqueCount="986">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1371" uniqueCount="988">
   <si>
     <t>id</t>
   </si>
@@ -3110,12 +3132,18 @@
   <si>
     <t>No sugar or insulin needed, keep automatic notification on to watch for any changes</t>
   </si>
+  <si>
+    <t>Word counts</t>
+  </si>
+  <si>
+    <t>Word counts:</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <fonts count="12">
+  <fonts count="13">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -3196,6 +3224,12 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -3217,7 +3251,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="19">
+  <borders count="26">
     <border>
       <left/>
       <right/>
@@ -3489,11 +3523,94 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FF284E3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF284E3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFF8F9FA"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFFFFFFF"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFFFFFFF"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -3590,11 +3707,69 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="4">
+  <dxfs count="5">
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <name val="&quot;Aptos Narrow&quot;"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FF000000"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color rgb="FF000000"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF000000"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
     <dxf>
       <border diagonalUp="0" diagonalDown="0">
         <right style="thin">
@@ -3630,9 +3805,9 @@
   </dxfs>
   <tableStyles count="1">
     <tableStyle name="Responses-style" pivot="0" count="3" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
-      <tableStyleElement type="headerRow" dxfId="3"/>
-      <tableStyleElement type="firstRowStripe" dxfId="2"/>
-      <tableStyleElement type="secondRowStripe" dxfId="1"/>
+      <tableStyleElement type="headerRow" dxfId="4"/>
+      <tableStyleElement type="firstRowStripe" dxfId="3"/>
+      <tableStyleElement type="secondRowStripe" dxfId="2"/>
     </tableStyle>
   </tableStyles>
   <extLst>
@@ -3647,9 +3822,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="All_responses" displayName="All_responses" ref="A1:S87">
-  <autoFilter ref="A1:S87" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
-  <tableColumns count="19">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="All_responses" displayName="All_responses" ref="A1:T87">
+  <autoFilter ref="A1:T87" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+  <tableColumns count="20">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="id"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Column 37"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Device"/>
@@ -3668,7 +3843,10 @@
     <tableColumn id="20" xr3:uid="{00000000-0010-0000-0000-000014000000}" name="Sensor error 2"/>
     <tableColumn id="21" xr3:uid="{00000000-0010-0000-0000-000015000000}" name="In range 1"/>
     <tableColumn id="22" xr3:uid="{00000000-0010-0000-0000-000016000000}" name="In range 2"/>
-    <tableColumn id="23" xr3:uid="{00000000-0010-0000-0000-000017000000}" name="Agree to text shown" dataDxfId="0"/>
+    <tableColumn id="6" xr3:uid="{758634FB-E90D-9247-9927-D2CFE67B979E}" name="Word counts" dataDxfId="0">
+      <calculatedColumnFormula array="1">SUMPRODUCT(IF(TRIM(E2:R2)="", 0, LEN(TRIM(E2:R2))-LEN(SUBSTITUTE(TRIM(E2:R2)," ",""))+1))</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="23" xr3:uid="{00000000-0010-0000-0000-000017000000}" name="Agree to text shown" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="Responses-style" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3875,7 +4053,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:S1004"/>
+  <dimension ref="A1:T1004"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="5.83203125" hidden="1" customWidth="1"/>
@@ -3888,10 +4066,11 @@
     <col min="13" max="13" width="23.5" customWidth="1"/>
     <col min="14" max="14" width="24.1640625" customWidth="1"/>
     <col min="15" max="18" width="37.6640625" customWidth="1"/>
-    <col min="19" max="19" width="25.1640625" style="35" customWidth="1"/>
+    <col min="19" max="19" width="9.1640625" customWidth="1"/>
+    <col min="20" max="20" width="25.1640625" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" ht="14" customHeight="1">
+    <row r="1" spans="1:20" ht="14" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3946,11 +4125,14 @@
       <c r="R1" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="29" t="s">
+      <c r="S1" s="36" t="s">
+        <v>986</v>
+      </c>
+      <c r="T1" s="29" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:19" ht="13">
+    <row r="2" spans="1:20" ht="13">
       <c r="A2" s="10">
         <v>12</v>
       </c>
@@ -3999,11 +4181,15 @@
       <c r="R2" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="S2" s="30" t="s">
+      <c r="S2" s="37" cm="1">
+        <f t="array" ref="S2">SUMPRODUCT(IF(TRIM(E2:R2)="", 0, LEN(TRIM(E2:R2))-LEN(SUBSTITUTE(TRIM(E2:R2)," ",""))+1))</f>
+        <v>51</v>
+      </c>
+      <c r="T2" s="30" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="3" spans="1:19" ht="13">
+    <row r="3" spans="1:20" ht="13">
       <c r="A3" s="7">
         <v>13</v>
       </c>
@@ -4052,11 +4238,15 @@
       <c r="R3" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="S3" s="31" t="s">
+      <c r="S3" s="38" cm="1">
+        <f t="array" ref="S3">SUMPRODUCT(IF(TRIM(E3:R3)="", 0, LEN(TRIM(E3:R3))-LEN(SUBSTITUTE(TRIM(E3:R3)," ",""))+1))</f>
+        <v>107</v>
+      </c>
+      <c r="T3" s="31" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="4" spans="1:19" ht="13">
+    <row r="4" spans="1:20" ht="13">
       <c r="A4" s="10">
         <v>14</v>
       </c>
@@ -4105,11 +4295,15 @@
       <c r="R4" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="S4" s="30" t="s">
+      <c r="S4" s="37" cm="1">
+        <f t="array" ref="S4">SUMPRODUCT(IF(TRIM(E4:R4)="", 0, LEN(TRIM(E4:R4))-LEN(SUBSTITUTE(TRIM(E4:R4)," ",""))+1))</f>
+        <v>414</v>
+      </c>
+      <c r="T4" s="30" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="5" spans="1:19" ht="13">
+    <row r="5" spans="1:20" ht="13">
       <c r="A5" s="7">
         <v>15</v>
       </c>
@@ -4158,11 +4352,15 @@
       <c r="R5" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="S5" s="31" t="s">
+      <c r="S5" s="38" cm="1">
+        <f t="array" ref="S5">SUMPRODUCT(IF(TRIM(E5:R5)="", 0, LEN(TRIM(E5:R5))-LEN(SUBSTITUTE(TRIM(E5:R5)," ",""))+1))</f>
+        <v>487</v>
+      </c>
+      <c r="T5" s="31" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="6" spans="1:19" ht="13">
+    <row r="6" spans="1:20" ht="13">
       <c r="A6" s="10">
         <v>16</v>
       </c>
@@ -4211,11 +4409,15 @@
       <c r="R6" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="S6" s="30" t="s">
+      <c r="S6" s="37" cm="1">
+        <f t="array" ref="S6">SUMPRODUCT(IF(TRIM(E6:R6)="", 0, LEN(TRIM(E6:R6))-LEN(SUBSTITUTE(TRIM(E6:R6)," ",""))+1))</f>
+        <v>68</v>
+      </c>
+      <c r="T6" s="30" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:19" ht="13">
+    <row r="7" spans="1:20" ht="13">
       <c r="A7" s="7">
         <v>17</v>
       </c>
@@ -4264,11 +4466,15 @@
       <c r="R7" s="9" t="s">
         <v>97</v>
       </c>
-      <c r="S7" s="31" t="s">
+      <c r="S7" s="38" cm="1">
+        <f t="array" ref="S7">SUMPRODUCT(IF(TRIM(E7:R7)="", 0, LEN(TRIM(E7:R7))-LEN(SUBSTITUTE(TRIM(E7:R7)," ",""))+1))</f>
+        <v>190</v>
+      </c>
+      <c r="T7" s="31" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="8" spans="1:19" ht="13">
+    <row r="8" spans="1:20" ht="13">
       <c r="A8" s="10">
         <v>18</v>
       </c>
@@ -4317,11 +4523,15 @@
       <c r="R8" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="S8" s="30" t="s">
+      <c r="S8" s="37" cm="1">
+        <f t="array" ref="S8">SUMPRODUCT(IF(TRIM(E8:R8)="", 0, LEN(TRIM(E8:R8))-LEN(SUBSTITUTE(TRIM(E8:R8)," ",""))+1))</f>
+        <v>214</v>
+      </c>
+      <c r="T8" s="30" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="9" spans="1:19" ht="13">
+    <row r="9" spans="1:20" ht="13">
       <c r="A9" s="7">
         <v>19</v>
       </c>
@@ -4370,11 +4580,15 @@
       <c r="R9" s="9" t="s">
         <v>119</v>
       </c>
-      <c r="S9" s="31" t="s">
+      <c r="S9" s="38" cm="1">
+        <f t="array" ref="S9">SUMPRODUCT(IF(TRIM(E9:R9)="", 0, LEN(TRIM(E9:R9))-LEN(SUBSTITUTE(TRIM(E9:R9)," ",""))+1))</f>
+        <v>145</v>
+      </c>
+      <c r="T9" s="31" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="10" spans="1:19" ht="13">
+    <row r="10" spans="1:20" ht="13">
       <c r="A10" s="10">
         <v>20</v>
       </c>
@@ -4423,11 +4637,15 @@
       <c r="R10" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="S10" s="30" t="s">
+      <c r="S10" s="37" cm="1">
+        <f t="array" ref="S10">SUMPRODUCT(IF(TRIM(E10:R10)="", 0, LEN(TRIM(E10:R10))-LEN(SUBSTITUTE(TRIM(E10:R10)," ",""))+1))</f>
+        <v>102</v>
+      </c>
+      <c r="T10" s="30" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="11" spans="1:19" ht="13">
+    <row r="11" spans="1:20" ht="13">
       <c r="A11" s="7">
         <v>21</v>
       </c>
@@ -4476,11 +4694,15 @@
       <c r="R11" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="S11" s="31" t="s">
+      <c r="S11" s="38" cm="1">
+        <f t="array" ref="S11">SUMPRODUCT(IF(TRIM(E11:R11)="", 0, LEN(TRIM(E11:R11))-LEN(SUBSTITUTE(TRIM(E11:R11)," ",""))+1))</f>
+        <v>343</v>
+      </c>
+      <c r="T11" s="31" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:19" ht="13">
+    <row r="12" spans="1:20" ht="13">
       <c r="A12" s="10">
         <v>22</v>
       </c>
@@ -4529,11 +4751,15 @@
       <c r="R12" s="12" t="s">
         <v>146</v>
       </c>
-      <c r="S12" s="30" t="s">
+      <c r="S12" s="37" cm="1">
+        <f t="array" ref="S12">SUMPRODUCT(IF(TRIM(E12:R12)="", 0, LEN(TRIM(E12:R12))-LEN(SUBSTITUTE(TRIM(E12:R12)," ",""))+1))</f>
+        <v>413</v>
+      </c>
+      <c r="T12" s="30" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="13" spans="1:19" ht="13">
+    <row r="13" spans="1:20" ht="13">
       <c r="A13" s="7">
         <v>23</v>
       </c>
@@ -4582,11 +4808,15 @@
       <c r="R13" s="9" t="s">
         <v>158</v>
       </c>
-      <c r="S13" s="31" t="s">
+      <c r="S13" s="38" cm="1">
+        <f t="array" ref="S13">SUMPRODUCT(IF(TRIM(E13:R13)="", 0, LEN(TRIM(E13:R13))-LEN(SUBSTITUTE(TRIM(E13:R13)," ",""))+1))</f>
+        <v>764</v>
+      </c>
+      <c r="T13" s="31" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="14" spans="1:19" ht="13">
+    <row r="14" spans="1:20" ht="13">
       <c r="A14" s="10">
         <v>24</v>
       </c>
@@ -4635,11 +4865,15 @@
       <c r="R14" s="12" t="s">
         <v>167</v>
       </c>
-      <c r="S14" s="30" t="s">
+      <c r="S14" s="37" cm="1">
+        <f t="array" ref="S14">SUMPRODUCT(IF(TRIM(E14:R14)="", 0, LEN(TRIM(E14:R14))-LEN(SUBSTITUTE(TRIM(E14:R14)," ",""))+1))</f>
+        <v>1199</v>
+      </c>
+      <c r="T14" s="30" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="15" spans="1:19" ht="13">
+    <row r="15" spans="1:20" ht="13">
       <c r="A15" s="7">
         <v>25</v>
       </c>
@@ -4688,11 +4922,15 @@
       <c r="R15" s="9" t="s">
         <v>181</v>
       </c>
-      <c r="S15" s="31" t="s">
+      <c r="S15" s="38" cm="1">
+        <f t="array" ref="S15">SUMPRODUCT(IF(TRIM(E15:R15)="", 0, LEN(TRIM(E15:R15))-LEN(SUBSTITUTE(TRIM(E15:R15)," ",""))+1))</f>
+        <v>288</v>
+      </c>
+      <c r="T15" s="31" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="16" spans="1:19" ht="13">
+    <row r="16" spans="1:20" ht="13">
       <c r="A16" s="10">
         <v>26</v>
       </c>
@@ -4741,11 +4979,15 @@
       <c r="R16" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="S16" s="30" t="s">
+      <c r="S16" s="37" cm="1">
+        <f t="array" ref="S16">SUMPRODUCT(IF(TRIM(E16:R16)="", 0, LEN(TRIM(E16:R16))-LEN(SUBSTITUTE(TRIM(E16:R16)," ",""))+1))</f>
+        <v>405</v>
+      </c>
+      <c r="T16" s="30" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="17" spans="1:19" ht="13">
+    <row r="17" spans="1:20" ht="13">
       <c r="A17" s="7">
         <v>27</v>
       </c>
@@ -4794,11 +5036,15 @@
       <c r="R17" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="S17" s="31" t="s">
+      <c r="S17" s="38" cm="1">
+        <f t="array" ref="S17">SUMPRODUCT(IF(TRIM(E17:R17)="", 0, LEN(TRIM(E17:R17))-LEN(SUBSTITUTE(TRIM(E17:R17)," ",""))+1))</f>
+        <v>46</v>
+      </c>
+      <c r="T17" s="31" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="18" spans="1:19" ht="13">
+    <row r="18" spans="1:20" ht="13">
       <c r="A18" s="10">
         <v>28</v>
       </c>
@@ -4851,11 +5097,15 @@
       <c r="R18" s="12" t="s">
         <v>211</v>
       </c>
-      <c r="S18" s="30" t="s">
+      <c r="S18" s="37" cm="1">
+        <f t="array" ref="S18">SUMPRODUCT(IF(TRIM(E18:R18)="", 0, LEN(TRIM(E18:R18))-LEN(SUBSTITUTE(TRIM(E18:R18)," ",""))+1))</f>
+        <v>224</v>
+      </c>
+      <c r="T18" s="30" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="19" spans="1:19" ht="13">
+    <row r="19" spans="1:20" ht="13">
       <c r="A19" s="7">
         <v>29</v>
       </c>
@@ -4904,11 +5154,15 @@
       <c r="R19" s="9" t="s">
         <v>223</v>
       </c>
-      <c r="S19" s="31" t="s">
+      <c r="S19" s="38" cm="1">
+        <f t="array" ref="S19">SUMPRODUCT(IF(TRIM(E19:R19)="", 0, LEN(TRIM(E19:R19))-LEN(SUBSTITUTE(TRIM(E19:R19)," ",""))+1))</f>
+        <v>149</v>
+      </c>
+      <c r="T19" s="31" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="20" spans="1:19" ht="13">
+    <row r="20" spans="1:20" ht="13">
       <c r="A20" s="10">
         <v>30</v>
       </c>
@@ -4961,11 +5215,15 @@
       <c r="R20" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="S20" s="30" t="s">
+      <c r="S20" s="37" cm="1">
+        <f t="array" ref="S20">SUMPRODUCT(IF(TRIM(E20:R20)="", 0, LEN(TRIM(E20:R20))-LEN(SUBSTITUTE(TRIM(E20:R20)," ",""))+1))</f>
+        <v>91</v>
+      </c>
+      <c r="T20" s="30" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="21" spans="1:19" ht="13">
+    <row r="21" spans="1:20" ht="13">
       <c r="A21" s="7">
         <v>31</v>
       </c>
@@ -5014,11 +5272,15 @@
       <c r="R21" s="9" t="s">
         <v>243</v>
       </c>
-      <c r="S21" s="31" t="s">
+      <c r="S21" s="38" cm="1">
+        <f t="array" ref="S21">SUMPRODUCT(IF(TRIM(E21:R21)="", 0, LEN(TRIM(E21:R21))-LEN(SUBSTITUTE(TRIM(E21:R21)," ",""))+1))</f>
+        <v>145</v>
+      </c>
+      <c r="T21" s="31" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="22" spans="1:19" ht="13">
+    <row r="22" spans="1:20" ht="13">
       <c r="A22" s="10">
         <v>32</v>
       </c>
@@ -5071,11 +5333,15 @@
       <c r="R22" s="12" t="s">
         <v>257</v>
       </c>
-      <c r="S22" s="30" t="s">
+      <c r="S22" s="37" cm="1">
+        <f t="array" ref="S22">SUMPRODUCT(IF(TRIM(E22:R22)="", 0, LEN(TRIM(E22:R22))-LEN(SUBSTITUTE(TRIM(E22:R22)," ",""))+1))</f>
+        <v>442</v>
+      </c>
+      <c r="T22" s="30" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="23" spans="1:19" ht="13">
+    <row r="23" spans="1:20" ht="13">
       <c r="A23" s="7">
         <v>33</v>
       </c>
@@ -5124,11 +5390,15 @@
       <c r="R23" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="S23" s="31" t="s">
+      <c r="S23" s="38" cm="1">
+        <f t="array" ref="S23">SUMPRODUCT(IF(TRIM(E23:R23)="", 0, LEN(TRIM(E23:R23))-LEN(SUBSTITUTE(TRIM(E23:R23)," ",""))+1))</f>
+        <v>109</v>
+      </c>
+      <c r="T23" s="31" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="24" spans="1:19" ht="13">
+    <row r="24" spans="1:20" ht="13">
       <c r="A24" s="10">
         <v>34</v>
       </c>
@@ -5177,11 +5447,15 @@
       <c r="R24" s="12" t="s">
         <v>280</v>
       </c>
-      <c r="S24" s="30" t="s">
+      <c r="S24" s="37" cm="1">
+        <f t="array" ref="S24">SUMPRODUCT(IF(TRIM(E24:R24)="", 0, LEN(TRIM(E24:R24))-LEN(SUBSTITUTE(TRIM(E24:R24)," ",""))+1))</f>
+        <v>103</v>
+      </c>
+      <c r="T24" s="30" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="25" spans="1:19" ht="13">
+    <row r="25" spans="1:20" ht="13">
       <c r="A25" s="7">
         <v>35</v>
       </c>
@@ -5230,11 +5504,15 @@
       <c r="R25" s="9" t="s">
         <v>291</v>
       </c>
-      <c r="S25" s="31" t="s">
+      <c r="S25" s="38" cm="1">
+        <f t="array" ref="S25">SUMPRODUCT(IF(TRIM(E25:R25)="", 0, LEN(TRIM(E25:R25))-LEN(SUBSTITUTE(TRIM(E25:R25)," ",""))+1))</f>
+        <v>83</v>
+      </c>
+      <c r="T25" s="31" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="26" spans="1:19" ht="13">
+    <row r="26" spans="1:20" ht="13">
       <c r="A26" s="10">
         <v>36</v>
       </c>
@@ -5283,11 +5561,15 @@
       <c r="R26" s="12" t="s">
         <v>303</v>
       </c>
-      <c r="S26" s="30" t="s">
+      <c r="S26" s="37" cm="1">
+        <f t="array" ref="S26">SUMPRODUCT(IF(TRIM(E26:R26)="", 0, LEN(TRIM(E26:R26))-LEN(SUBSTITUTE(TRIM(E26:R26)," ",""))+1))</f>
+        <v>154</v>
+      </c>
+      <c r="T26" s="30" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="27" spans="1:19" ht="13">
+    <row r="27" spans="1:20" ht="13">
       <c r="A27" s="7">
         <v>37</v>
       </c>
@@ -5340,11 +5622,15 @@
       <c r="R27" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="S27" s="31" t="s">
+      <c r="S27" s="38" cm="1">
+        <f t="array" ref="S27">SUMPRODUCT(IF(TRIM(E27:R27)="", 0, LEN(TRIM(E27:R27))-LEN(SUBSTITUTE(TRIM(E27:R27)," ",""))+1))</f>
+        <v>402</v>
+      </c>
+      <c r="T27" s="31" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="28" spans="1:19" ht="13">
+    <row r="28" spans="1:20" ht="13">
       <c r="A28" s="10">
         <v>38</v>
       </c>
@@ -5397,11 +5683,15 @@
       <c r="R28" s="12" t="s">
         <v>327</v>
       </c>
-      <c r="S28" s="30" t="s">
+      <c r="S28" s="37" cm="1">
+        <f t="array" ref="S28">SUMPRODUCT(IF(TRIM(E28:R28)="", 0, LEN(TRIM(E28:R28))-LEN(SUBSTITUTE(TRIM(E28:R28)," ",""))+1))</f>
+        <v>788</v>
+      </c>
+      <c r="T28" s="30" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="29" spans="1:19" ht="13">
+    <row r="29" spans="1:20" ht="13">
       <c r="A29" s="7">
         <v>39</v>
       </c>
@@ -5450,11 +5740,15 @@
       <c r="R29" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="S29" s="31" t="s">
+      <c r="S29" s="38" cm="1">
+        <f t="array" ref="S29">SUMPRODUCT(IF(TRIM(E29:R29)="", 0, LEN(TRIM(E29:R29))-LEN(SUBSTITUTE(TRIM(E29:R29)," ",""))+1))</f>
+        <v>236</v>
+      </c>
+      <c r="T29" s="31" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="30" spans="1:19" ht="13">
+    <row r="30" spans="1:20" ht="13">
       <c r="A30" s="10">
         <v>40</v>
       </c>
@@ -5507,11 +5801,15 @@
       <c r="R30" s="12" t="s">
         <v>351</v>
       </c>
-      <c r="S30" s="30" t="s">
+      <c r="S30" s="37" cm="1">
+        <f t="array" ref="S30">SUMPRODUCT(IF(TRIM(E30:R30)="", 0, LEN(TRIM(E30:R30))-LEN(SUBSTITUTE(TRIM(E30:R30)," ",""))+1))</f>
+        <v>378</v>
+      </c>
+      <c r="T30" s="30" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="31" spans="1:19" ht="13">
+    <row r="31" spans="1:20" ht="13">
       <c r="A31" s="7">
         <v>41</v>
       </c>
@@ -5560,11 +5858,15 @@
       <c r="R31" s="9" t="s">
         <v>363</v>
       </c>
-      <c r="S31" s="31" t="s">
+      <c r="S31" s="38" cm="1">
+        <f t="array" ref="S31">SUMPRODUCT(IF(TRIM(E31:R31)="", 0, LEN(TRIM(E31:R31))-LEN(SUBSTITUTE(TRIM(E31:R31)," ",""))+1))</f>
+        <v>445</v>
+      </c>
+      <c r="T31" s="31" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="32" spans="1:19" ht="13">
+    <row r="32" spans="1:20" ht="13">
       <c r="A32" s="10">
         <v>42</v>
       </c>
@@ -5613,11 +5915,15 @@
       <c r="R32" s="12" t="s">
         <v>374</v>
       </c>
-      <c r="S32" s="30" t="s">
+      <c r="S32" s="37" cm="1">
+        <f t="array" ref="S32">SUMPRODUCT(IF(TRIM(E32:R32)="", 0, LEN(TRIM(E32:R32))-LEN(SUBSTITUTE(TRIM(E32:R32)," ",""))+1))</f>
+        <v>344</v>
+      </c>
+      <c r="T32" s="30" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="33" spans="1:19" ht="13">
+    <row r="33" spans="1:20" ht="13">
       <c r="A33" s="7">
         <v>43</v>
       </c>
@@ -5670,11 +5976,15 @@
       <c r="R33" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="S33" s="31" t="s">
+      <c r="S33" s="38" cm="1">
+        <f t="array" ref="S33">SUMPRODUCT(IF(TRIM(E33:R33)="", 0, LEN(TRIM(E33:R33))-LEN(SUBSTITUTE(TRIM(E33:R33)," ",""))+1))</f>
+        <v>176</v>
+      </c>
+      <c r="T33" s="31" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="34" spans="1:19" ht="13">
+    <row r="34" spans="1:20" ht="13">
       <c r="A34" s="10">
         <v>44</v>
       </c>
@@ -5723,11 +6033,15 @@
       <c r="R34" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="S34" s="30" t="s">
+      <c r="S34" s="37" cm="1">
+        <f t="array" ref="S34">SUMPRODUCT(IF(TRIM(E34:R34)="", 0, LEN(TRIM(E34:R34))-LEN(SUBSTITUTE(TRIM(E34:R34)," ",""))+1))</f>
+        <v>50</v>
+      </c>
+      <c r="T34" s="30" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="35" spans="1:19" ht="13">
+    <row r="35" spans="1:20" ht="13">
       <c r="A35" s="7">
         <v>45</v>
       </c>
@@ -5780,11 +6094,15 @@
       <c r="R35" s="9" t="s">
         <v>407</v>
       </c>
-      <c r="S35" s="31" t="s">
+      <c r="S35" s="38" cm="1">
+        <f t="array" ref="S35">SUMPRODUCT(IF(TRIM(E35:R35)="", 0, LEN(TRIM(E35:R35))-LEN(SUBSTITUTE(TRIM(E35:R35)," ",""))+1))</f>
+        <v>368</v>
+      </c>
+      <c r="T35" s="31" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="36" spans="1:19" ht="13">
+    <row r="36" spans="1:20" ht="13">
       <c r="A36" s="10">
         <v>46</v>
       </c>
@@ -5833,11 +6151,15 @@
       <c r="R36" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="S36" s="30" t="s">
+      <c r="S36" s="37" cm="1">
+        <f t="array" ref="S36">SUMPRODUCT(IF(TRIM(E36:R36)="", 0, LEN(TRIM(E36:R36))-LEN(SUBSTITUTE(TRIM(E36:R36)," ",""))+1))</f>
+        <v>59</v>
+      </c>
+      <c r="T36" s="30" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="37" spans="1:19" ht="13">
+    <row r="37" spans="1:20" ht="13">
       <c r="A37" s="7">
         <v>47</v>
       </c>
@@ -5890,11 +6212,15 @@
       <c r="R37" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="S37" s="31" t="s">
+      <c r="S37" s="38" cm="1">
+        <f t="array" ref="S37">SUMPRODUCT(IF(TRIM(E37:R37)="", 0, LEN(TRIM(E37:R37))-LEN(SUBSTITUTE(TRIM(E37:R37)," ",""))+1))</f>
+        <v>62</v>
+      </c>
+      <c r="T37" s="31" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="38" spans="1:19" ht="13">
+    <row r="38" spans="1:20" ht="13">
       <c r="A38" s="10">
         <v>48</v>
       </c>
@@ -5943,11 +6269,15 @@
       <c r="R38" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="S38" s="30" t="s">
+      <c r="S38" s="37" cm="1">
+        <f t="array" ref="S38">SUMPRODUCT(IF(TRIM(E38:R38)="", 0, LEN(TRIM(E38:R38))-LEN(SUBSTITUTE(TRIM(E38:R38)," ",""))+1))</f>
+        <v>300</v>
+      </c>
+      <c r="T38" s="30" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="39" spans="1:19" ht="13">
+    <row r="39" spans="1:20" ht="13">
       <c r="A39" s="7">
         <v>49</v>
       </c>
@@ -6000,11 +6330,15 @@
       <c r="R39" s="9" t="s">
         <v>450</v>
       </c>
-      <c r="S39" s="31" t="s">
+      <c r="S39" s="38" cm="1">
+        <f t="array" ref="S39">SUMPRODUCT(IF(TRIM(E39:R39)="", 0, LEN(TRIM(E39:R39))-LEN(SUBSTITUTE(TRIM(E39:R39)," ",""))+1))</f>
+        <v>890</v>
+      </c>
+      <c r="T39" s="31" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="40" spans="1:19" ht="13">
+    <row r="40" spans="1:20" ht="13">
       <c r="A40" s="10">
         <v>50</v>
       </c>
@@ -6053,11 +6387,15 @@
       <c r="R40" s="12" t="s">
         <v>461</v>
       </c>
-      <c r="S40" s="30" t="s">
+      <c r="S40" s="37" cm="1">
+        <f t="array" ref="S40">SUMPRODUCT(IF(TRIM(E40:R40)="", 0, LEN(TRIM(E40:R40))-LEN(SUBSTITUTE(TRIM(E40:R40)," ",""))+1))</f>
+        <v>127</v>
+      </c>
+      <c r="T40" s="30" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="41" spans="1:19" ht="13">
+    <row r="41" spans="1:20" ht="13">
       <c r="A41" s="7">
         <v>51</v>
       </c>
@@ -6106,11 +6444,15 @@
       <c r="R41" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="S41" s="31" t="s">
+      <c r="S41" s="38" cm="1">
+        <f t="array" ref="S41">SUMPRODUCT(IF(TRIM(E41:R41)="", 0, LEN(TRIM(E41:R41))-LEN(SUBSTITUTE(TRIM(E41:R41)," ",""))+1))</f>
+        <v>38</v>
+      </c>
+      <c r="T41" s="31" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="42" spans="1:19" ht="13">
+    <row r="42" spans="1:20" ht="13">
       <c r="A42" s="10">
         <v>52</v>
       </c>
@@ -6163,11 +6505,15 @@
       <c r="R42" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="S42" s="30" t="s">
+      <c r="S42" s="37" cm="1">
+        <f t="array" ref="S42">SUMPRODUCT(IF(TRIM(E42:R42)="", 0, LEN(TRIM(E42:R42))-LEN(SUBSTITUTE(TRIM(E42:R42)," ",""))+1))</f>
+        <v>80</v>
+      </c>
+      <c r="T42" s="30" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="43" spans="1:19" ht="13">
+    <row r="43" spans="1:20" ht="13">
       <c r="A43" s="7">
         <v>53</v>
       </c>
@@ -6220,11 +6566,15 @@
       <c r="R43" s="9" t="s">
         <v>490</v>
       </c>
-      <c r="S43" s="31" t="s">
+      <c r="S43" s="38" cm="1">
+        <f t="array" ref="S43">SUMPRODUCT(IF(TRIM(E43:R43)="", 0, LEN(TRIM(E43:R43))-LEN(SUBSTITUTE(TRIM(E43:R43)," ",""))+1))</f>
+        <v>306</v>
+      </c>
+      <c r="T43" s="31" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="44" spans="1:19" ht="13">
+    <row r="44" spans="1:20" ht="13">
       <c r="A44" s="10">
         <v>54</v>
       </c>
@@ -6273,11 +6623,15 @@
       <c r="R44" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="S44" s="30" t="s">
+      <c r="S44" s="37" cm="1">
+        <f t="array" ref="S44">SUMPRODUCT(IF(TRIM(E44:R44)="", 0, LEN(TRIM(E44:R44))-LEN(SUBSTITUTE(TRIM(E44:R44)," ",""))+1))</f>
+        <v>154</v>
+      </c>
+      <c r="T44" s="30" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="45" spans="1:19" ht="13">
+    <row r="45" spans="1:20" ht="13">
       <c r="A45" s="7">
         <v>55</v>
       </c>
@@ -6326,11 +6680,15 @@
       <c r="R45" s="9" t="s">
         <v>512</v>
       </c>
-      <c r="S45" s="31" t="s">
+      <c r="S45" s="38" cm="1">
+        <f t="array" ref="S45">SUMPRODUCT(IF(TRIM(E45:R45)="", 0, LEN(TRIM(E45:R45))-LEN(SUBSTITUTE(TRIM(E45:R45)," ",""))+1))</f>
+        <v>451</v>
+      </c>
+      <c r="T45" s="31" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="46" spans="1:19" ht="13">
+    <row r="46" spans="1:20" ht="13">
       <c r="A46" s="10">
         <v>56</v>
       </c>
@@ -6383,11 +6741,15 @@
       <c r="R46" s="12" t="s">
         <v>526</v>
       </c>
-      <c r="S46" s="30" t="s">
+      <c r="S46" s="37" cm="1">
+        <f t="array" ref="S46">SUMPRODUCT(IF(TRIM(E46:R46)="", 0, LEN(TRIM(E46:R46))-LEN(SUBSTITUTE(TRIM(E46:R46)," ",""))+1))</f>
+        <v>257</v>
+      </c>
+      <c r="T46" s="30" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="47" spans="1:19" ht="13">
+    <row r="47" spans="1:20" ht="13">
       <c r="A47" s="7">
         <v>57</v>
       </c>
@@ -6436,11 +6798,15 @@
       <c r="R47" s="9" t="s">
         <v>535</v>
       </c>
-      <c r="S47" s="31" t="s">
+      <c r="S47" s="38" cm="1">
+        <f t="array" ref="S47">SUMPRODUCT(IF(TRIM(E47:R47)="", 0, LEN(TRIM(E47:R47))-LEN(SUBSTITUTE(TRIM(E47:R47)," ",""))+1))</f>
+        <v>110</v>
+      </c>
+      <c r="T47" s="31" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="48" spans="1:19" ht="13">
+    <row r="48" spans="1:20" ht="13">
       <c r="A48" s="10">
         <v>58</v>
       </c>
@@ -6489,11 +6855,15 @@
       <c r="R48" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="S48" s="30" t="s">
+      <c r="S48" s="37" cm="1">
+        <f t="array" ref="S48">SUMPRODUCT(IF(TRIM(E48:R48)="", 0, LEN(TRIM(E48:R48))-LEN(SUBSTITUTE(TRIM(E48:R48)," ",""))+1))</f>
+        <v>221</v>
+      </c>
+      <c r="T48" s="30" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="49" spans="1:19" ht="13">
+    <row r="49" spans="1:20" ht="13">
       <c r="A49" s="7">
         <v>59</v>
       </c>
@@ -6546,11 +6916,15 @@
       <c r="R49" s="9" t="s">
         <v>559</v>
       </c>
-      <c r="S49" s="32" t="s">
+      <c r="S49" s="39" cm="1">
+        <f t="array" ref="S49">SUMPRODUCT(IF(TRIM(E49:R49)="", 0, LEN(TRIM(E49:R49))-LEN(SUBSTITUTE(TRIM(E49:R49)," ",""))+1))</f>
+        <v>74</v>
+      </c>
+      <c r="T49" s="32" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="50" spans="1:19" ht="13">
+    <row r="50" spans="1:20" ht="13">
       <c r="A50" s="10">
         <v>60</v>
       </c>
@@ -6603,11 +6977,15 @@
       <c r="R50" s="20" t="s">
         <v>568</v>
       </c>
-      <c r="S50" s="33" t="s">
+      <c r="S50" s="40" cm="1">
+        <f t="array" ref="S50">SUMPRODUCT(IF(TRIM(E50:R50)="", 0, LEN(TRIM(E50:R50))-LEN(SUBSTITUTE(TRIM(E50:R50)," ",""))+1))</f>
+        <v>82</v>
+      </c>
+      <c r="T50" s="33" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="51" spans="1:19" ht="13">
+    <row r="51" spans="1:20" ht="13">
       <c r="A51" s="7">
         <v>61</v>
       </c>
@@ -6660,11 +7038,15 @@
       <c r="R51" s="20" t="s">
         <v>582</v>
       </c>
-      <c r="S51" s="33" t="s">
+      <c r="S51" s="40" cm="1">
+        <f t="array" ref="S51">SUMPRODUCT(IF(TRIM(E51:R51)="", 0, LEN(TRIM(E51:R51))-LEN(SUBSTITUTE(TRIM(E51:R51)," ",""))+1))</f>
+        <v>287</v>
+      </c>
+      <c r="T51" s="33" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="52" spans="1:19" ht="13">
+    <row r="52" spans="1:20" ht="13">
       <c r="A52" s="10">
         <v>62</v>
       </c>
@@ -6713,11 +7095,15 @@
       <c r="R52" s="20" t="s">
         <v>594</v>
       </c>
-      <c r="S52" s="33" t="s">
+      <c r="S52" s="40" cm="1">
+        <f t="array" ref="S52">SUMPRODUCT(IF(TRIM(E52:R52)="", 0, LEN(TRIM(E52:R52))-LEN(SUBSTITUTE(TRIM(E52:R52)," ",""))+1))</f>
+        <v>432</v>
+      </c>
+      <c r="T52" s="33" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="53" spans="1:19" ht="13">
+    <row r="53" spans="1:20" ht="13">
       <c r="A53" s="7">
         <v>63</v>
       </c>
@@ -6766,11 +7152,15 @@
       <c r="R53" s="20" t="s">
         <v>606</v>
       </c>
-      <c r="S53" s="33" t="s">
+      <c r="S53" s="40" cm="1">
+        <f t="array" ref="S53">SUMPRODUCT(IF(TRIM(E53:R53)="", 0, LEN(TRIM(E53:R53))-LEN(SUBSTITUTE(TRIM(E53:R53)," ",""))+1))</f>
+        <v>250</v>
+      </c>
+      <c r="T53" s="33" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="54" spans="1:19" ht="13">
+    <row r="54" spans="1:20" ht="13">
       <c r="A54" s="10">
         <v>64</v>
       </c>
@@ -6819,11 +7209,15 @@
       <c r="R54" s="20" t="s">
         <v>37</v>
       </c>
-      <c r="S54" s="33" t="s">
+      <c r="S54" s="40" cm="1">
+        <f t="array" ref="S54">SUMPRODUCT(IF(TRIM(E54:R54)="", 0, LEN(TRIM(E54:R54))-LEN(SUBSTITUTE(TRIM(E54:R54)," ",""))+1))</f>
+        <v>95</v>
+      </c>
+      <c r="T54" s="33" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="55" spans="1:19" ht="13">
+    <row r="55" spans="1:20" ht="13">
       <c r="A55" s="7">
         <v>65</v>
       </c>
@@ -6876,11 +7270,15 @@
       <c r="R55" s="20" t="s">
         <v>558</v>
       </c>
-      <c r="S55" s="33" t="s">
+      <c r="S55" s="40" cm="1">
+        <f t="array" ref="S55">SUMPRODUCT(IF(TRIM(E55:R55)="", 0, LEN(TRIM(E55:R55))-LEN(SUBSTITUTE(TRIM(E55:R55)," ",""))+1))</f>
+        <v>93</v>
+      </c>
+      <c r="T55" s="33" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="56" spans="1:19" ht="13">
+    <row r="56" spans="1:20" ht="13">
       <c r="A56" s="10">
         <v>66</v>
       </c>
@@ -6933,11 +7331,15 @@
       <c r="R56" s="20" t="s">
         <v>37</v>
       </c>
-      <c r="S56" s="33" t="s">
+      <c r="S56" s="40" cm="1">
+        <f t="array" ref="S56">SUMPRODUCT(IF(TRIM(E56:R56)="", 0, LEN(TRIM(E56:R56))-LEN(SUBSTITUTE(TRIM(E56:R56)," ",""))+1))</f>
+        <v>263</v>
+      </c>
+      <c r="T56" s="33" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="57" spans="1:19" ht="13">
+    <row r="57" spans="1:20" ht="13">
       <c r="A57" s="7">
         <v>67</v>
       </c>
@@ -6986,11 +7388,15 @@
       <c r="R57" s="20" t="s">
         <v>654</v>
       </c>
-      <c r="S57" s="33" t="s">
+      <c r="S57" s="40" cm="1">
+        <f t="array" ref="S57">SUMPRODUCT(IF(TRIM(E57:R57)="", 0, LEN(TRIM(E57:R57))-LEN(SUBSTITUTE(TRIM(E57:R57)," ",""))+1))</f>
+        <v>98</v>
+      </c>
+      <c r="T57" s="33" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="58" spans="1:19" ht="13">
+    <row r="58" spans="1:20" ht="13">
       <c r="A58" s="10">
         <v>68</v>
       </c>
@@ -7039,11 +7445,15 @@
       <c r="R58" s="20" t="s">
         <v>37</v>
       </c>
-      <c r="S58" s="33" t="s">
+      <c r="S58" s="40" cm="1">
+        <f t="array" ref="S58">SUMPRODUCT(IF(TRIM(E58:R58)="", 0, LEN(TRIM(E58:R58))-LEN(SUBSTITUTE(TRIM(E58:R58)," ",""))+1))</f>
+        <v>135</v>
+      </c>
+      <c r="T58" s="33" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="59" spans="1:19" ht="13">
+    <row r="59" spans="1:20" ht="13">
       <c r="A59" s="7">
         <v>69</v>
       </c>
@@ -7092,11 +7502,15 @@
       <c r="R59" s="20" t="s">
         <v>674</v>
       </c>
-      <c r="S59" s="33" t="s">
+      <c r="S59" s="40" cm="1">
+        <f t="array" ref="S59">SUMPRODUCT(IF(TRIM(E59:R59)="", 0, LEN(TRIM(E59:R59))-LEN(SUBSTITUTE(TRIM(E59:R59)," ",""))+1))</f>
+        <v>81</v>
+      </c>
+      <c r="T59" s="33" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="60" spans="1:19" ht="13">
+    <row r="60" spans="1:20" ht="13">
       <c r="A60" s="10">
         <v>70</v>
       </c>
@@ -7149,11 +7563,15 @@
       <c r="R60" s="20" t="s">
         <v>688</v>
       </c>
-      <c r="S60" s="33" t="s">
+      <c r="S60" s="40" cm="1">
+        <f t="array" ref="S60">SUMPRODUCT(IF(TRIM(E60:R60)="", 0, LEN(TRIM(E60:R60))-LEN(SUBSTITUTE(TRIM(E60:R60)," ",""))+1))</f>
+        <v>254</v>
+      </c>
+      <c r="T60" s="33" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="61" spans="1:19" ht="13">
+    <row r="61" spans="1:20" ht="13">
       <c r="A61" s="7">
         <v>71</v>
       </c>
@@ -7202,11 +7620,15 @@
       <c r="R61" s="20" t="s">
         <v>699</v>
       </c>
-      <c r="S61" s="33" t="s">
+      <c r="S61" s="40" cm="1">
+        <f t="array" ref="S61">SUMPRODUCT(IF(TRIM(E61:R61)="", 0, LEN(TRIM(E61:R61))-LEN(SUBSTITUTE(TRIM(E61:R61)," ",""))+1))</f>
+        <v>87</v>
+      </c>
+      <c r="T61" s="33" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="62" spans="1:19" ht="13">
+    <row r="62" spans="1:20" ht="13">
       <c r="A62" s="10">
         <v>72</v>
       </c>
@@ -7255,11 +7677,15 @@
       <c r="R62" s="20" t="s">
         <v>708</v>
       </c>
-      <c r="S62" s="33" t="s">
+      <c r="S62" s="40" cm="1">
+        <f t="array" ref="S62">SUMPRODUCT(IF(TRIM(E62:R62)="", 0, LEN(TRIM(E62:R62))-LEN(SUBSTITUTE(TRIM(E62:R62)," ",""))+1))</f>
+        <v>104</v>
+      </c>
+      <c r="T62" s="33" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="63" spans="1:19" ht="13">
+    <row r="63" spans="1:20" ht="13">
       <c r="A63" s="7">
         <v>73</v>
       </c>
@@ -7312,11 +7738,15 @@
       <c r="R63" s="20" t="s">
         <v>37</v>
       </c>
-      <c r="S63" s="33" t="s">
+      <c r="S63" s="40" cm="1">
+        <f t="array" ref="S63">SUMPRODUCT(IF(TRIM(E63:R63)="", 0, LEN(TRIM(E63:R63))-LEN(SUBSTITUTE(TRIM(E63:R63)," ",""))+1))</f>
+        <v>106</v>
+      </c>
+      <c r="T63" s="33" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="64" spans="1:19" ht="13">
+    <row r="64" spans="1:20" ht="13">
       <c r="A64" s="10">
         <v>74</v>
       </c>
@@ -7365,11 +7795,15 @@
       <c r="R64" s="20" t="s">
         <v>37</v>
       </c>
-      <c r="S64" s="33" t="s">
+      <c r="S64" s="40" cm="1">
+        <f t="array" ref="S64">SUMPRODUCT(IF(TRIM(E64:R64)="", 0, LEN(TRIM(E64:R64))-LEN(SUBSTITUTE(TRIM(E64:R64)," ",""))+1))</f>
+        <v>47</v>
+      </c>
+      <c r="T64" s="33" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="65" spans="1:19" ht="13">
+    <row r="65" spans="1:20" ht="13">
       <c r="A65" s="7">
         <v>75</v>
       </c>
@@ -7418,11 +7852,15 @@
       <c r="R65" s="20" t="s">
         <v>37</v>
       </c>
-      <c r="S65" s="33" t="s">
+      <c r="S65" s="40" cm="1">
+        <f t="array" ref="S65">SUMPRODUCT(IF(TRIM(E65:R65)="", 0, LEN(TRIM(E65:R65))-LEN(SUBSTITUTE(TRIM(E65:R65)," ",""))+1))</f>
+        <v>132</v>
+      </c>
+      <c r="T65" s="33" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="66" spans="1:19" ht="13">
+    <row r="66" spans="1:20" ht="13">
       <c r="A66" s="10">
         <v>76</v>
       </c>
@@ -7471,11 +7909,15 @@
       <c r="R66" s="20" t="s">
         <v>37</v>
       </c>
-      <c r="S66" s="33" t="s">
+      <c r="S66" s="40" cm="1">
+        <f t="array" ref="S66">SUMPRODUCT(IF(TRIM(E66:R66)="", 0, LEN(TRIM(E66:R66))-LEN(SUBSTITUTE(TRIM(E66:R66)," ",""))+1))</f>
+        <v>68</v>
+      </c>
+      <c r="T66" s="33" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="67" spans="1:19" ht="13">
+    <row r="67" spans="1:20" ht="13">
       <c r="A67" s="7">
         <v>77</v>
       </c>
@@ -7524,11 +7966,15 @@
       <c r="R67" s="20" t="s">
         <v>37</v>
       </c>
-      <c r="S67" s="33" t="s">
+      <c r="S67" s="40" cm="1">
+        <f t="array" ref="S67">SUMPRODUCT(IF(TRIM(E67:R67)="", 0, LEN(TRIM(E67:R67))-LEN(SUBSTITUTE(TRIM(E67:R67)," ",""))+1))</f>
+        <v>210</v>
+      </c>
+      <c r="T67" s="33" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="68" spans="1:19" ht="13">
+    <row r="68" spans="1:20" ht="13">
       <c r="A68" s="10">
         <v>78</v>
       </c>
@@ -7581,11 +8027,15 @@
       <c r="R68" s="20" t="s">
         <v>37</v>
       </c>
-      <c r="S68" s="33" t="s">
+      <c r="S68" s="40" cm="1">
+        <f t="array" ref="S68">SUMPRODUCT(IF(TRIM(E68:R68)="", 0, LEN(TRIM(E68:R68))-LEN(SUBSTITUTE(TRIM(E68:R68)," ",""))+1))</f>
+        <v>48</v>
+      </c>
+      <c r="T68" s="33" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="69" spans="1:19" ht="13">
+    <row r="69" spans="1:20" ht="13">
       <c r="A69" s="7">
         <v>79</v>
       </c>
@@ -7638,11 +8088,15 @@
       <c r="R69" s="20" t="s">
         <v>37</v>
       </c>
-      <c r="S69" s="33" t="s">
+      <c r="S69" s="40" cm="1">
+        <f t="array" ref="S69">SUMPRODUCT(IF(TRIM(E69:R69)="", 0, LEN(TRIM(E69:R69))-LEN(SUBSTITUTE(TRIM(E69:R69)," ",""))+1))</f>
+        <v>146</v>
+      </c>
+      <c r="T69" s="33" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="70" spans="1:19" ht="13">
+    <row r="70" spans="1:20" ht="13">
       <c r="A70" s="10">
         <v>80</v>
       </c>
@@ -7695,11 +8149,15 @@
       <c r="R70" s="20" t="s">
         <v>37</v>
       </c>
-      <c r="S70" s="33" t="s">
+      <c r="S70" s="40" cm="1">
+        <f t="array" ref="S70">SUMPRODUCT(IF(TRIM(E70:R70)="", 0, LEN(TRIM(E70:R70))-LEN(SUBSTITUTE(TRIM(E70:R70)," ",""))+1))</f>
+        <v>199</v>
+      </c>
+      <c r="T70" s="33" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="71" spans="1:19" ht="13">
+    <row r="71" spans="1:20" ht="13">
       <c r="A71" s="7">
         <v>81</v>
       </c>
@@ -7748,11 +8206,15 @@
       <c r="R71" s="20" t="s">
         <v>708</v>
       </c>
-      <c r="S71" s="33" t="s">
+      <c r="S71" s="40" cm="1">
+        <f t="array" ref="S71">SUMPRODUCT(IF(TRIM(E71:R71)="", 0, LEN(TRIM(E71:R71))-LEN(SUBSTITUTE(TRIM(E71:R71)," ",""))+1))</f>
+        <v>196</v>
+      </c>
+      <c r="T71" s="33" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="72" spans="1:19" ht="13">
+    <row r="72" spans="1:20" ht="13">
       <c r="A72" s="10">
         <v>82</v>
       </c>
@@ -7805,11 +8267,15 @@
       <c r="R72" s="20" t="s">
         <v>37</v>
       </c>
-      <c r="S72" s="33" t="s">
+      <c r="S72" s="40" cm="1">
+        <f t="array" ref="S72">SUMPRODUCT(IF(TRIM(E72:R72)="", 0, LEN(TRIM(E72:R72))-LEN(SUBSTITUTE(TRIM(E72:R72)," ",""))+1))</f>
+        <v>326</v>
+      </c>
+      <c r="T72" s="33" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="73" spans="1:19" ht="13">
+    <row r="73" spans="1:20" ht="13">
       <c r="A73" s="7">
         <v>83</v>
       </c>
@@ -7862,11 +8328,15 @@
       <c r="R73" s="20" t="s">
         <v>37</v>
       </c>
-      <c r="S73" s="33" t="s">
+      <c r="S73" s="40" cm="1">
+        <f t="array" ref="S73">SUMPRODUCT(IF(TRIM(E73:R73)="", 0, LEN(TRIM(E73:R73))-LEN(SUBSTITUTE(TRIM(E73:R73)," ",""))+1))</f>
+        <v>110</v>
+      </c>
+      <c r="T73" s="33" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="74" spans="1:19" ht="13">
+    <row r="74" spans="1:20" ht="13">
       <c r="A74" s="10">
         <v>84</v>
       </c>
@@ -7919,11 +8389,15 @@
       <c r="R74" s="20" t="s">
         <v>37</v>
       </c>
-      <c r="S74" s="33" t="s">
+      <c r="S74" s="40" cm="1">
+        <f t="array" ref="S74">SUMPRODUCT(IF(TRIM(E74:R74)="", 0, LEN(TRIM(E74:R74))-LEN(SUBSTITUTE(TRIM(E74:R74)," ",""))+1))</f>
+        <v>147</v>
+      </c>
+      <c r="T74" s="33" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="75" spans="1:19" ht="13">
+    <row r="75" spans="1:20" ht="13">
       <c r="A75" s="7">
         <v>85</v>
       </c>
@@ -7976,11 +8450,15 @@
       <c r="R75" s="20" t="s">
         <v>851</v>
       </c>
-      <c r="S75" s="33" t="s">
+      <c r="S75" s="40" cm="1">
+        <f t="array" ref="S75">SUMPRODUCT(IF(TRIM(E75:R75)="", 0, LEN(TRIM(E75:R75))-LEN(SUBSTITUTE(TRIM(E75:R75)," ",""))+1))</f>
+        <v>226</v>
+      </c>
+      <c r="T75" s="33" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="76" spans="1:19" ht="13">
+    <row r="76" spans="1:20" ht="13">
       <c r="A76" s="10">
         <v>86</v>
       </c>
@@ -8029,11 +8507,15 @@
       <c r="R76" s="20" t="s">
         <v>861</v>
       </c>
-      <c r="S76" s="33" t="s">
+      <c r="S76" s="40" cm="1">
+        <f t="array" ref="S76">SUMPRODUCT(IF(TRIM(E76:R76)="", 0, LEN(TRIM(E76:R76))-LEN(SUBSTITUTE(TRIM(E76:R76)," ",""))+1))</f>
+        <v>70</v>
+      </c>
+      <c r="T76" s="33" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="77" spans="1:19" ht="13">
+    <row r="77" spans="1:20" ht="13">
       <c r="A77" s="7">
         <v>87</v>
       </c>
@@ -8082,11 +8564,15 @@
       <c r="R77" s="20" t="s">
         <v>37</v>
       </c>
-      <c r="S77" s="33" t="s">
+      <c r="S77" s="40" cm="1">
+        <f t="array" ref="S77">SUMPRODUCT(IF(TRIM(E77:R77)="", 0, LEN(TRIM(E77:R77))-LEN(SUBSTITUTE(TRIM(E77:R77)," ",""))+1))</f>
+        <v>79</v>
+      </c>
+      <c r="T77" s="33" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="78" spans="1:19" ht="13">
+    <row r="78" spans="1:20" ht="13">
       <c r="A78" s="10">
         <v>88</v>
       </c>
@@ -8139,11 +8625,15 @@
       <c r="R78" s="20" t="s">
         <v>37</v>
       </c>
-      <c r="S78" s="33" t="s">
+      <c r="S78" s="40" cm="1">
+        <f t="array" ref="S78">SUMPRODUCT(IF(TRIM(E78:R78)="", 0, LEN(TRIM(E78:R78))-LEN(SUBSTITUTE(TRIM(E78:R78)," ",""))+1))</f>
+        <v>146</v>
+      </c>
+      <c r="T78" s="33" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="79" spans="1:19" ht="13">
+    <row r="79" spans="1:20" ht="13">
       <c r="A79" s="7">
         <v>89</v>
       </c>
@@ -8192,11 +8682,15 @@
       <c r="R79" s="20" t="s">
         <v>37</v>
       </c>
-      <c r="S79" s="33" t="s">
+      <c r="S79" s="40" cm="1">
+        <f t="array" ref="S79">SUMPRODUCT(IF(TRIM(E79:R79)="", 0, LEN(TRIM(E79:R79))-LEN(SUBSTITUTE(TRIM(E79:R79)," ",""))+1))</f>
+        <v>85</v>
+      </c>
+      <c r="T79" s="33" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="80" spans="1:19" ht="13">
+    <row r="80" spans="1:20" ht="13">
       <c r="A80" s="10">
         <v>90</v>
       </c>
@@ -8249,11 +8743,15 @@
       <c r="R80" s="20" t="s">
         <v>37</v>
       </c>
-      <c r="S80" s="33" t="s">
+      <c r="S80" s="40" cm="1">
+        <f t="array" ref="S80">SUMPRODUCT(IF(TRIM(E80:R80)="", 0, LEN(TRIM(E80:R80))-LEN(SUBSTITUTE(TRIM(E80:R80)," ",""))+1))</f>
+        <v>138</v>
+      </c>
+      <c r="T80" s="33" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="81" spans="1:19" ht="13">
+    <row r="81" spans="1:20" ht="13">
       <c r="A81" s="7">
         <v>91</v>
       </c>
@@ -8302,11 +8800,15 @@
       <c r="R81" s="20" t="s">
         <v>37</v>
       </c>
-      <c r="S81" s="33" t="s">
+      <c r="S81" s="40" cm="1">
+        <f t="array" ref="S81">SUMPRODUCT(IF(TRIM(E81:R81)="", 0, LEN(TRIM(E81:R81))-LEN(SUBSTITUTE(TRIM(E81:R81)," ",""))+1))</f>
+        <v>240</v>
+      </c>
+      <c r="T81" s="33" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="82" spans="1:19" ht="13">
+    <row r="82" spans="1:20" ht="13">
       <c r="A82" s="10">
         <v>92</v>
       </c>
@@ -8355,11 +8857,15 @@
       <c r="R82" s="20" t="s">
         <v>927</v>
       </c>
-      <c r="S82" s="33" t="s">
+      <c r="S82" s="40" cm="1">
+        <f t="array" ref="S82">SUMPRODUCT(IF(TRIM(E82:R82)="", 0, LEN(TRIM(E82:R82))-LEN(SUBSTITUTE(TRIM(E82:R82)," ",""))+1))</f>
+        <v>147</v>
+      </c>
+      <c r="T82" s="33" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="83" spans="1:19" ht="13">
+    <row r="83" spans="1:20" ht="13">
       <c r="A83" s="7">
         <v>93</v>
       </c>
@@ -8408,11 +8914,15 @@
       <c r="R83" s="20" t="s">
         <v>938</v>
       </c>
-      <c r="S83" s="33" t="s">
+      <c r="S83" s="40" cm="1">
+        <f t="array" ref="S83">SUMPRODUCT(IF(TRIM(E83:R83)="", 0, LEN(TRIM(E83:R83))-LEN(SUBSTITUTE(TRIM(E83:R83)," ",""))+1))</f>
+        <v>96</v>
+      </c>
+      <c r="T83" s="33" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="84" spans="1:19" ht="13">
+    <row r="84" spans="1:20" ht="13">
       <c r="A84" s="10">
         <v>94</v>
       </c>
@@ -8465,11 +8975,15 @@
       <c r="R84" s="20" t="s">
         <v>37</v>
       </c>
-      <c r="S84" s="33" t="s">
+      <c r="S84" s="40" cm="1">
+        <f t="array" ref="S84">SUMPRODUCT(IF(TRIM(E84:R84)="", 0, LEN(TRIM(E84:R84))-LEN(SUBSTITUTE(TRIM(E84:R84)," ",""))+1))</f>
+        <v>159</v>
+      </c>
+      <c r="T84" s="33" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="85" spans="1:19" ht="13">
+    <row r="85" spans="1:20" ht="13">
       <c r="A85" s="7">
         <v>95</v>
       </c>
@@ -8518,11 +9032,15 @@
       <c r="R85" s="20" t="s">
         <v>961</v>
       </c>
-      <c r="S85" s="33" t="s">
+      <c r="S85" s="40" cm="1">
+        <f t="array" ref="S85">SUMPRODUCT(IF(TRIM(E85:R85)="", 0, LEN(TRIM(E85:R85))-LEN(SUBSTITUTE(TRIM(E85:R85)," ",""))+1))</f>
+        <v>88</v>
+      </c>
+      <c r="T85" s="33" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="86" spans="1:19" ht="13">
+    <row r="86" spans="1:20" ht="13">
       <c r="A86" s="10">
         <v>96</v>
       </c>
@@ -8571,106 +9089,159 @@
       <c r="R86" s="20" t="s">
         <v>973</v>
       </c>
-      <c r="S86" s="33" t="s">
+      <c r="S86" s="40" cm="1">
+        <f t="array" ref="S86">SUMPRODUCT(IF(TRIM(E86:R86)="", 0, LEN(TRIM(E86:R86))-LEN(SUBSTITUTE(TRIM(E86:R86)," ",""))+1))</f>
+        <v>228</v>
+      </c>
+      <c r="T86" s="33" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="87" spans="1:19" ht="13">
+    <row r="87" spans="1:20" ht="13">
       <c r="A87" s="23">
         <v>97</v>
       </c>
       <c r="B87" s="24"/>
-      <c r="C87" s="19" t="s">
+      <c r="C87" s="41" t="s">
         <v>27</v>
       </c>
-      <c r="D87" s="19" t="s">
+      <c r="D87" s="41" t="s">
         <v>19</v>
       </c>
-      <c r="E87" s="20" t="s">
+      <c r="E87" s="42" t="s">
         <v>974</v>
       </c>
-      <c r="F87" s="20" t="s">
+      <c r="F87" s="42" t="s">
         <v>975</v>
       </c>
-      <c r="G87" s="20" t="s">
+      <c r="G87" s="42" t="s">
         <v>976</v>
       </c>
-      <c r="H87" s="20" t="s">
+      <c r="H87" s="42" t="s">
         <v>977</v>
       </c>
-      <c r="I87" s="20" t="s">
+      <c r="I87" s="42" t="s">
         <v>978</v>
       </c>
-      <c r="J87" s="20" t="s">
+      <c r="J87" s="42" t="s">
         <v>979</v>
       </c>
-      <c r="K87" s="20" t="s">
+      <c r="K87" s="42" t="s">
         <v>980</v>
       </c>
-      <c r="L87" s="20" t="s">
+      <c r="L87" s="42" t="s">
         <v>981</v>
       </c>
-      <c r="M87" s="20"/>
-      <c r="N87" s="20"/>
-      <c r="O87" s="20" t="s">
+      <c r="M87" s="42"/>
+      <c r="N87" s="42"/>
+      <c r="O87" s="42" t="s">
         <v>982</v>
       </c>
-      <c r="P87" s="20" t="s">
+      <c r="P87" s="42" t="s">
         <v>983</v>
       </c>
-      <c r="Q87" s="20" t="s">
+      <c r="Q87" s="42" t="s">
         <v>984</v>
       </c>
-      <c r="R87" s="20" t="s">
+      <c r="R87" s="42" t="s">
         <v>985</v>
       </c>
-      <c r="S87" s="33" t="s">
+      <c r="S87" s="40" cm="1">
+        <f t="array" ref="S87">SUMPRODUCT(IF(TRIM(E87:R87)="", 0, LEN(TRIM(E87:R87))-LEN(SUBSTITUTE(TRIM(E87:R87)," ",""))+1))</f>
+        <v>146</v>
+      </c>
+      <c r="T87" s="33" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="88" spans="1:19" ht="13">
+    <row r="88" spans="1:20" ht="13">
       <c r="A88" s="25"/>
       <c r="B88" s="26"/>
-      <c r="C88" s="26"/>
-      <c r="D88" s="26"/>
-      <c r="E88" s="26"/>
-      <c r="F88" s="26"/>
-      <c r="G88" s="26"/>
-      <c r="H88" s="26"/>
-      <c r="I88" s="26"/>
-      <c r="J88" s="26"/>
-      <c r="K88" s="26"/>
-      <c r="L88" s="26"/>
-      <c r="M88" s="26"/>
-      <c r="N88" s="26"/>
-      <c r="O88" s="26"/>
-      <c r="P88" s="26"/>
-      <c r="Q88" s="26"/>
-      <c r="R88" s="26"/>
-      <c r="S88" s="34"/>
-    </row>
-    <row r="89" spans="1:19" ht="13">
+      <c r="C88" s="43" t="s">
+        <v>987</v>
+      </c>
+      <c r="D88" s="43"/>
+      <c r="E88" s="44" cm="1">
+        <f t="array" ref="E88">SUMPRODUCT(IF(TRIM(E2:E87)="", 0, LEN(TRIM(E2:E87))-LEN(SUBSTITUTE(TRIM(E2:E87)," ",""))+1))</f>
+        <v>1405</v>
+      </c>
+      <c r="F88" s="44" cm="1">
+        <f t="array" ref="F88">SUMPRODUCT(IF(TRIM(F2:F87)="", 0, LEN(TRIM(F2:F87))-LEN(SUBSTITUTE(TRIM(F2:F87)," ",""))+1))</f>
+        <v>1470</v>
+      </c>
+      <c r="G88" s="44" cm="1">
+        <f t="array" ref="G88">SUMPRODUCT(IF(TRIM(G2:G87)="", 0, LEN(TRIM(G2:G87))-LEN(SUBSTITUTE(TRIM(G2:G87)," ",""))+1))</f>
+        <v>1327</v>
+      </c>
+      <c r="H88" s="44" cm="1">
+        <f t="array" ref="H88">SUMPRODUCT(IF(TRIM(H2:H87)="", 0, LEN(TRIM(H2:H87))-LEN(SUBSTITUTE(TRIM(H2:H87)," ",""))+1))</f>
+        <v>2050</v>
+      </c>
+      <c r="I88" s="44" cm="1">
+        <f t="array" ref="I88">SUMPRODUCT(IF(TRIM(I2:I87)="", 0, LEN(TRIM(I2:I87))-LEN(SUBSTITUTE(TRIM(I2:I87)," ",""))+1))</f>
+        <v>2325</v>
+      </c>
+      <c r="J88" s="44" cm="1">
+        <f t="array" ref="J88">SUMPRODUCT(IF(TRIM(J2:J87)="", 0, LEN(TRIM(J2:J87))-LEN(SUBSTITUTE(TRIM(J2:J87)," ",""))+1))</f>
+        <v>1867</v>
+      </c>
+      <c r="K88" s="44" cm="1">
+        <f t="array" ref="K88">SUMPRODUCT(IF(TRIM(K2:K87)="", 0, LEN(TRIM(K2:K87))-LEN(SUBSTITUTE(TRIM(K2:K87)," ",""))+1))</f>
+        <v>1419</v>
+      </c>
+      <c r="L88" s="44" cm="1">
+        <f t="array" ref="L88">SUMPRODUCT(IF(TRIM(L2:L87)="", 0, LEN(TRIM(L2:L87))-LEN(SUBSTITUTE(TRIM(L2:L87)," ",""))+1))</f>
+        <v>1459</v>
+      </c>
+      <c r="M88" s="44" cm="1">
+        <f t="array" ref="M88">SUMPRODUCT(IF(TRIM(M2:M87)="", 0, LEN(TRIM(M2:M87))-LEN(SUBSTITUTE(TRIM(M2:M87)," ",""))+1))</f>
+        <v>425</v>
+      </c>
+      <c r="N88" s="44" cm="1">
+        <f t="array" ref="N88">SUMPRODUCT(IF(TRIM(N2:N87)="", 0, LEN(TRIM(N2:N87))-LEN(SUBSTITUTE(TRIM(N2:N87)," ",""))+1))</f>
+        <v>483</v>
+      </c>
+      <c r="O88" s="44" cm="1">
+        <f t="array" ref="O88">SUMPRODUCT(IF(TRIM(O2:O87)="", 0, LEN(TRIM(O2:O87))-LEN(SUBSTITUTE(TRIM(O2:O87)," ",""))+1))</f>
+        <v>1482</v>
+      </c>
+      <c r="P88" s="44" cm="1">
+        <f t="array" ref="P88">SUMPRODUCT(IF(TRIM(P2:P87)="", 0, LEN(TRIM(P2:P87))-LEN(SUBSTITUTE(TRIM(P2:P87)," ",""))+1))</f>
+        <v>1662</v>
+      </c>
+      <c r="Q88" s="44" cm="1">
+        <f t="array" ref="Q88">SUMPRODUCT(IF(TRIM(Q2:Q87)="", 0, LEN(TRIM(Q2:Q87))-LEN(SUBSTITUTE(TRIM(Q2:Q87)," ",""))+1))</f>
+        <v>824</v>
+      </c>
+      <c r="R88" s="44" cm="1">
+        <f t="array" ref="R88">SUMPRODUCT(IF(TRIM(R2:R87)="", 0, LEN(TRIM(R2:R87))-LEN(SUBSTITUTE(TRIM(R2:R87)," ",""))+1))</f>
+        <v>698</v>
+      </c>
+      <c r="S88" s="26"/>
+      <c r="T88" s="34"/>
+    </row>
+    <row r="89" spans="1:20" ht="13">
       <c r="A89" s="25"/>
     </row>
-    <row r="90" spans="1:19" ht="13">
+    <row r="90" spans="1:20" ht="13">
       <c r="A90" s="25"/>
     </row>
-    <row r="91" spans="1:19" ht="13">
+    <row r="91" spans="1:20" ht="13">
       <c r="A91" s="25"/>
     </row>
-    <row r="92" spans="1:19" ht="13">
+    <row r="92" spans="1:20" ht="13">
       <c r="A92" s="25"/>
     </row>
-    <row r="93" spans="1:19" ht="13">
+    <row r="93" spans="1:20" ht="13">
       <c r="A93" s="25"/>
     </row>
-    <row r="94" spans="1:19" ht="13">
+    <row r="94" spans="1:20" ht="13">
       <c r="A94" s="25"/>
     </row>
-    <row r="95" spans="1:19" ht="13">
+    <row r="95" spans="1:20" ht="13">
       <c r="A95" s="25"/>
     </row>
-    <row r="96" spans="1:19" ht="13">
+    <row r="96" spans="1:20" ht="13">
       <c r="A96" s="25"/>
     </row>
     <row r="97" spans="1:6" ht="26.25" customHeight="1">
@@ -11401,11 +11972,15 @@
       <c r="A1004" s="25"/>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="C88:D88"/>
+  </mergeCells>
+  <phoneticPr fontId="12" type="noConversion"/>
   <dataValidations count="3">
     <dataValidation type="list" allowBlank="1" sqref="D2:D87" xr:uid="{00000000-0002-0000-0000-000004000000}">
       <formula1>"Baseline,Meaning"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="S2:S87" xr:uid="{00000000-0002-0000-0000-000005000000}">
+    <dataValidation type="list" allowBlank="1" sqref="T2:T87" xr:uid="{00000000-0002-0000-0000-000005000000}">
       <formula1>"Agree,Strongly agree,Neither,Disagree,Somewhat disagree,Somewhat agree,Strongly disagree"</formula1>
     </dataValidation>
     <dataValidation allowBlank="1" showDropDown="1" sqref="C2:C87" xr:uid="{00000000-0002-0000-0000-000008000000}"/>

</xml_diff>